<commit_message>
Add August WhatsApp IT correspondence to MoFA Log - August 2026
Adds 24 IT items from the MOFA Content WhatsApp chat (IT sheet now 62 rows),
August-only after review.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TGjTRH6W5gZfxXYUTY19k1
</commit_message>
<xml_diff>
--- a/output/MoFA Log - August2026 Final.xlsx
+++ b/output/MoFA Log - August2026 Final.xlsx
@@ -18232,7 +18232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G64"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="5" min="1" max="1"/>
@@ -18424,24 +18424,102 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="351" customHeight="1">
+    <row r="6" ht="336" customHeight="1">
       <c r="A6" s="7" t="n">
         <v>4</v>
       </c>
       <c r="B6" s="8" t="n">
+        <v>46237</v>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Request to Revert Changes – Hide "Category" Field on the Top Universities Page</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srini
+Thank you for your continued support.
+We kindly request that you revert all the changes made based on the request below regarding hiding the "Category" field on the Top Universities page.
+It appears that the changes implemented as part of this request may have caused the current issue. If possible, could you please roll back all the modifications and restore the website to its previous state, where everything was functioning correctly?
+The request we are referring to is:
+* Request: Hide the "Category" field on the Top Universities page.
+* Scope: Hide the field from the frontend only, while keeping it available in the CMS.
+* CMS Path: /sitecore/content/LDSC/Global/Top Universities Updated/TOP
+We would greatly appreciate your assistance in restoring the previous version so that we can continue investigating the issue from our side.
+(Confirmed path to point to: /sitecore/content/LDSC/Global/Top Universities Updated)</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="7" t="n"/>
+    </row>
+    <row r="7" ht="381" customHeight="1">
+      <c r="A7" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>46237</v>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Top Universities Page – Hide Specialty &amp; Sub Category Columns and Update the Second Filter</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Based on the meeting with Carla, we kindly request your assistance in implementing the following changes:
+Page URL:
+https://mofastg.mofaic.gov.ae/en/top-universities
+CMS Path:
+/sitecore/content/LDSC/Global/Top Universities Updated
+Request 1:
+Please hide (not delete) the Specialty and Sub Category columns from the table displayed on the frontend.
+After applying this change, the table should display only the following columns:
+* University
+* Country
+Please find the attached screenshot highlighting the two columns that need to be hidden.
+Request 2:
+The second filter currently displays values from both the Main Category and the Sub Category.
+The required behavior is for the second filter to display only the values from the Sub Category, located under the following CMS path:
+/sitecore/content/LDSC/Global/Lookups/Top Universities SubCategory
+The values from the Main Category should no longer appear in the second filter.</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>https://mofastg.mofaic.gov.ae/en/top-universities</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="351" customHeight="1">
+      <c r="A8" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="8" t="n">
         <v>46238</v>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>Issues Reported – Paris Mission Website (New Template)</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan
 The Paris Mission website has been created using the new missions template. Please find the Arabic version link below:
@@ -18457,31 +18535,31 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/missions/paris-new</t>
         </is>
       </c>
-      <c r="G6" s="7" t="n"/>
-    </row>
-    <row r="7" ht="156" customHeight="1">
-      <c r="A7" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" s="8" t="n">
+      <c r="G8" s="7" t="n"/>
+    </row>
+    <row r="9" ht="156" customHeight="1">
+      <c r="A9" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="8" t="n">
         <v>46238</v>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>Urgent Request to Hide the User Guide Video on the Attestation Page</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan
 Based on Enas's request from the Government Communication team, this is an urgent request to hide the User Guide video on the Attestation page.
@@ -18494,35 +18572,171 @@
 Please find the attached image for reference.</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/services/attestation</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="G9" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/en/services/attestation</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="351" customHeight="1">
-      <c r="A8" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" s="8" t="n">
+    <row r="10" ht="306" customHeight="1">
+      <c r="A10" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>46238</v>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Top Universities Page – Apply the Requested Changes to the Arabic Page (Urgent)</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Regarding the Top Universities page, the Government Communication team has informed us that the changes we recently sent should also be implemented on the following Arabic page.
+As this is an urgent request, we kindly ask you to prioritize its implementation.
+Page URL:
+https://mofastg.mofaic.gov.ae/ar-ae/top-universities
+Thank you for your prompt support.
+Kholoud informed us about the link you shared with us.
+We will get back to them and ask them to contact you directly through that link.
+Carla has just informed us that she has already contacted you and confirmed the page link we sent.
+Kindly proceed with implementing the requested changes as soon as possible, as this is an urgent request from the Government Communication team.
+Thank you very much for your continued support.</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>https://mofastg.mofaic.gov.ae/ar-ae/top-universities</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="n"/>
+    </row>
+    <row r="11" ht="216" customHeight="1">
+      <c r="A11" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>46238</v>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Top Universities Page – Request 1 (Hide Two Columns) Not Yet Implemented</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Thank you. However, it seems that only the second request has been completed.
+The first request, which was to hide the two columns from the page, has not been implemented yet.
+We need to hide the "Specialty" and "Sub Category" columns from the frontend page so that only the University and Country columns are displayed in the table, as requested.
+Could you please implement this change as well?
+Thank you for your support.
+Page URL: https://mofastg.mofaic.gov.ae/en/top-universities</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>https://mofastg.mofaic.gov.ae/en/top-universities</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="396" customHeight="1">
+      <c r="A12" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>46238</v>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Top Universities Page – Duplicate Records Displayed on the Frontend</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Note:
+We have also noticed that the content entered through the CMS is being duplicated on the frontend.
+Each university and its corresponding specialty has been entered only once in the CMS. However, the same records are appearing twice on the website.
+Example: For Canada under the Data Science specialty, there are three universities in the CMS, but they are displayed as six universities on the frontend due to duplication.
+Could you please investigate this issue as well?
+To resolve the duplication issue, we would like to remove the dependency on the Main Category and rely only on the Sub Category values configured in the CMS.
+The page should use only the Sub Category values stored in the CMS for filtering and displaying the universities. This should eliminate the duplicate records currently appearing on the frontend.
+In other words, please ignore the Main Category and use only the Sub Category in the page logic.
+What would you recommend as the best approach to resolve this issue?
+We would like to eliminate the duplicate records appearing on the frontend.
+We would appreciate your advice on the best way to permanently eliminate these duplicates.
+Thank you in advance for your support.</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="n"/>
+    </row>
+    <row r="13" ht="171" customHeight="1">
+      <c r="A13" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="8" t="n">
+        <v>46238</v>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Top Universities Page – No Results Displayed for Canada / Data Science After Recent Changes</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>Thank you for your efforts. The columns have now been successfully hidden.
+However, we have noticed another issue. When we search for Canada and select the Data Science specialty, no universities are displayed, even though there are three universities in the CMS that are classified under the Data Science subcategory.
+Could you please investigate this issue? It appears that the page is no longer retrieving the universities correctly after the recent changes.
+Thank you for your continued support.</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+    </row>
+    <row r="14" ht="351" customHeight="1">
+      <c r="A14" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="8" t="n">
         <v>46239</v>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t>500 Internal Server Error When Publishing News Items – Paris Mission</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E14" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 While publishing news articles for the Paris Mission, we encountered an issue where publishing certain news items causes a 500 Internal Server Error, making the entire News section unavailable.
@@ -18541,35 +18755,35 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/missions/_inprogress/paris</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/en/missions/_inprogress/paris</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="336" customHeight="1">
-      <c r="A9" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="B9" s="8" t="n">
+    <row r="15" ht="336" customHeight="1">
+      <c r="A15" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="8" t="n">
         <v>46239</v>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>Re: 500 Internal Server Error When Publishing News Items – Paris Mission</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E15" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 We would like to provide some additional information regarding the issue.
@@ -18583,27 +18797,166 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
-    </row>
-    <row r="10" ht="201" customHeight="1">
-      <c r="A10" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" s="8" t="n">
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="7" t="n"/>
+    </row>
+    <row r="16" ht="171" customHeight="1">
+      <c r="A16" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="8" t="n">
+        <v>46239</v>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Request to Hide the "Specialization" Filter on the Top Universities Page</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srini
+Based on a request from our colleagues in the Government Communication Department, we kindly ask for your support in hiding the third filter, "Specialization," from the Top Universities page.
+Page URL:
+https://mofastg.mofaic.gov.ae/en/top-universities
+Please find the attached screenshot for reference.
+Thank you in advance for your continued support.</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>https://mofastg.mofaic.gov.ae/en/top-universities</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="321" customHeight="1">
+      <c r="A17" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="8" t="n">
+        <v>46239</v>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>500 Error When Publishing Third-Language (French) News – Paris Mission</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srini
+We have identified an issue while publishing news for the Paris Mission, which is configured as a three-language website.
+When a news item exists only in the third language (French) and is published, the entire News section returns a 500 Internal Server Error.
+For example, the following news item reproduces the issue:
+Content Path:
+/sitecore/content/LDSC/Home/Missions/_Inprogress/paris/Media hub/News/paris-news
+If this item is published together with the other news items and the publishing targets include Arabic, English, and French, the entire News section becomes unavailable and displays a 500 Internal Server Error.
+Could you please investigate the root cause of this issue? It appears to be related to publishing news items that have content only in the third language.
+Thank you very much for your continued support and assistance.
+Page URL: https://www.mofa.gov.ae/en/missions/_inprogress/paris/media-hub/news</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="n"/>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/en/missions/_inprogress/paris/media-hub/news</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="186" customHeight="1">
+      <c r="A18" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="8" t="n">
+        <v>46239</v>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Language Switcher Not Redirecting to English – Cairo Mission Website</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>We would also like to inquire about another issue we encountered while migrating a new mission website.
+When changing the language on the Cairo Mission website from Arabic to English, the website still loads the Arabic version instead of redirecting to the corresponding English page.
+Website URL:
+https://www.mofa.gov.ae/Missions/_Inprogress/cairo
+Could you please investigate this issue and verify whether the language switcher is correctly configured for the new mission website?</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/Missions/_Inprogress/cairo</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="n"/>
+    </row>
+    <row r="19" ht="201" customHeight="1">
+      <c r="A19" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="8" t="n">
+        <v>46239</v>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Request for CMS Path of an Untranslated Label – Cairo Mission News Page</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>Could you please help us identify the CMS path for the label highlighted in red in the attached screenshot?
+We noticed that this label is still displayed in English on the Arabic version of the page, and we would like to locate its source in order to update the translation.
+Page URL:
+https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/cairo/Media-hub/News
+Please find the attached screenshot highlighting the label in question.
+We would appreciate your assistance in providing the corresponding CMS path.</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/cairo/Media-hub/News</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="n"/>
+    </row>
+    <row r="20" ht="201" customHeight="1">
+      <c r="A20" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="8" t="n">
         <v>46240</v>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>Re: 500 Internal Server Error When Publishing News Items – Paris Mission</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E20" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 Thank you very much for all the support and assistance you have provided. It is greatly appreciated.
@@ -18616,31 +18969,188 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/fr-fr/Missions/_Inprogress/paris</t>
         </is>
       </c>
-      <c r="G10" s="7" t="n"/>
-    </row>
-    <row r="11" ht="216" customHeight="1">
-      <c r="A11" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="B11" s="8" t="n">
+      <c r="G20" s="7" t="n"/>
+    </row>
+    <row r="21" ht="306" customHeight="1">
+      <c r="A21" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="8" t="n">
+        <v>46240</v>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Remaining Arabic Dictionary Entries – New Missions Websites</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>Regarding the words shown in the attached screenshots, we noticed that the path you shared does not include the required updates.
+These are the final remaining entries that need to be added to the Arabic dictionary. Once they are updated, the Arabic dictionary should be complete from our side.
+Thank you for your support, and please let us know once the updates have been applied.
+Sorry for the confusion regarding the paths I sent earlier.
+We tried using them, but it seems that some of the paths do not actually exist, while the others do not allow us to edit the content we need. It appears that there might be something incorrect with the paths provided.
+Could you please verify this for us?
+What we need are only the exact paths for the text labels highlighted in the attached screenshots, so that we can update those specific words directly.
+Thank you very much for your support and assistance.</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="n"/>
+      <c r="G21" s="7" t="n"/>
+    </row>
+    <row r="22" ht="201" customHeight="1">
+      <c r="A22" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="8" t="n">
+        <v>46240</v>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Baghdad Mission Website Migration Completed – Request to Test the News Rendering Script</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>Thank you very much for your continued support and assistance.
+The migration of the Baghdad Mission website has now been completed, and the site is available at the following link:
+https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Baghdad
+Could you please use this website to test the new script designed to automatically organize and display the news items correctly?
+Please let us know once the test has been completed, or if you need any additional information from our side.
+Thank you again for your support.</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Baghdad</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="n"/>
+    </row>
+    <row r="23" ht="201" customHeight="1">
+      <c r="A23" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="8" t="n">
+        <v>46240</v>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Arabic Labels (Embassy News / Embassy Statements) and Homepage Language Switching Check</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>Thank you for your support.
+The six terms have been fixed successfully. However, the following two items are still displaying incorrectly in Arabic:
+Embassy News (أخبار السفارة)
+Embassy Statements (بيانات السفارة)
+One last request, if possible, could you please also check the language switching functionality on the homepage? Specifically, when switching from Arabic to English and vice versa, to ensure everything is working correctly and the translations are displayed as expected.
+Thank you again for your continued support.</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="7" t="n"/>
+    </row>
+    <row r="24" ht="231" customHeight="1">
+      <c r="A24" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="8" t="n">
+        <v>46240</v>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Converting the Digital Attestation Page to the New Layout – Cairo Mission</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>Could you please help us with the Digital Attestation page? We would like to update it to match the new layout and design used on the current website.
+Page URL:
+https://www.mofa.gov.ae/Missions/_Inprogress/cairo/Services/Services-for-Individuals/Attestation-Information
+Is there a specific rendering, similar to the one used for the News pages, or any recommended approach that we should follow?
+We have already migrated the page from the old website to the new one; however, it is still retaining the old layout and styling.
+We would appreciate your guidance on the best way to convert it to the new design.</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/Missions/_Inprogress/cairo/Services/Services-for-Individuals/Attestation-Information</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="n"/>
+    </row>
+    <row r="25" ht="126" customHeight="1">
+      <c r="A25" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" s="8" t="n">
+        <v>46240</v>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>News Section Sorting – Display News by Publication Date (Newest First)</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>During our review of the website, we noticed an issue with the ordering of the News section. Currently, the news items are displayed in a random order.
+Could you please update the sorting logic so that news articles are displayed in descending order by publication date, with the most recent news appearing first, as implemented on the old website?
+Thank you for your support.</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="n"/>
+      <c r="G25" s="7" t="n"/>
+    </row>
+    <row r="26" ht="216" customHeight="1">
+      <c r="A26" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="8" t="n">
         <v>46242</v>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D26" s="7" t="inlineStr">
         <is>
           <t>Request to Migrate the News Section to the New Design – Doha Mission Website</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E26" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 Thank you very much for your continued support and assistance.
@@ -18654,31 +19164,31 @@
 Regards</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F26" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Doha/Media-hub/News</t>
         </is>
       </c>
-      <c r="G11" s="7" t="n"/>
-    </row>
-    <row r="12" ht="171" customHeight="1">
-      <c r="A12" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="B12" s="8" t="n">
+      <c r="G26" s="7" t="n"/>
+    </row>
+    <row r="27" ht="171" customHeight="1">
+      <c r="A27" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" s="8" t="n">
         <v>46243</v>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>Request to Upgrade the News Section to the New Design – Jeddah Mission Website</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E27" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 Thank you very much for your continued support and assistance.
@@ -18690,31 +19200,31 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="F27" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/Missions/_Inprogress/Jeddah/Media-hub/Embassy-News</t>
         </is>
       </c>
-      <c r="G12" s="7" t="n"/>
-    </row>
-    <row r="13" ht="231" customHeight="1">
-      <c r="A13" s="7" t="n">
-        <v>11</v>
-      </c>
-      <c r="B13" s="8" t="n">
+      <c r="G27" s="7" t="n"/>
+    </row>
+    <row r="28" ht="231" customHeight="1">
+      <c r="A28" s="7" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" s="8" t="n">
         <v>46243</v>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C28" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D28" s="7" t="inlineStr">
         <is>
           <t>Request to Migrate the News Section to the New Design – Algeria Mission Website</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E28" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 Thank you very much for your continuous support and assistance.
@@ -18728,31 +19238,31 @@
 Kind regards,</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F28" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Algeria/Media-hub/News</t>
         </is>
       </c>
-      <c r="G13" s="7" t="n"/>
-    </row>
-    <row r="14" ht="409" customHeight="1">
-      <c r="A14" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="B14" s="8" t="n">
+      <c r="G28" s="7" t="n"/>
+    </row>
+    <row r="29" ht="409" customHeight="1">
+      <c r="A29" s="7" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="8" t="n">
         <v>46243</v>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>Request to Update the News Section and Resolve the Media Center Display Issue – UAE Embassy in Jordan</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E29" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 Thank you very much for your continued support and assistance.
@@ -18776,31 +19286,31 @@
 (Attachments: Media Center -1.png, Media Center-2.png)</t>
         </is>
       </c>
-      <c r="F14" s="7" t="n"/>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="F29" s="7" t="n"/>
+      <c r="G29" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/en/Missions/_Inprogress/Amman</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="261" customHeight="1">
-      <c r="A15" s="7" t="n">
-        <v>13</v>
-      </c>
-      <c r="B15" s="8" t="n">
+    <row r="30" ht="261" customHeight="1">
+      <c r="A30" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" s="8" t="n">
         <v>46244</v>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C30" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D30" s="7" t="inlineStr">
         <is>
           <t>Request to Migrate the News Section to the New Template – Sofia Mission</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E30" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 Thank you very much for your continued support and assistance.
@@ -18815,31 +19325,31 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F30" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/missions/_inprogress/sofia/media-hub/news</t>
         </is>
       </c>
-      <c r="G15" s="7" t="n"/>
-    </row>
-    <row r="16" ht="261" customHeight="1">
-      <c r="A16" s="7" t="n">
-        <v>14</v>
-      </c>
-      <c r="B16" s="8" t="n">
+      <c r="G30" s="7" t="n"/>
+    </row>
+    <row r="31" ht="261" customHeight="1">
+      <c r="A31" s="7" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" s="8" t="n">
         <v>46244</v>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t>Request to Update the News Section Template – Tunis Mission Website</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E31" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 Thank you very much for your continued support and assistance.
@@ -18854,31 +19364,31 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F31" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/missions/_inprogress/tunis/media-hub/news</t>
         </is>
       </c>
-      <c r="G16" s="7" t="n"/>
-    </row>
-    <row r="17" ht="186" customHeight="1">
-      <c r="A17" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="B17" s="8" t="n">
+      <c r="G31" s="7" t="n"/>
+    </row>
+    <row r="32" ht="186" customHeight="1">
+      <c r="A32" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" s="8" t="n">
         <v>46244</v>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C32" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D32" s="7" t="inlineStr">
         <is>
           <t>Request to Move the Top Universities Page to Production</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="E32" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 Based on a request from Kholoud from the Government Communication Department,
@@ -18890,31 +19400,31 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F32" s="7" t="inlineStr">
         <is>
           <t>https://mofastg.mofaic.gov.ae/ar-ae/top-universities</t>
         </is>
       </c>
-      <c r="G17" s="7" t="n"/>
-    </row>
-    <row r="18" ht="291" customHeight="1">
-      <c r="A18" s="7" t="n">
-        <v>16</v>
-      </c>
-      <c r="B18" s="8" t="n">
+      <c r="G32" s="7" t="n"/>
+    </row>
+    <row r="33" ht="291" customHeight="1">
+      <c r="A33" s="7" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" s="8" t="n">
         <v>46244</v>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D33" s="7" t="inlineStr">
         <is>
           <t>Issue with Email Display on the Media Interview Request Page – Riyadh Mission</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E33" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 Thank you very much for your continued support and assistance.
@@ -18931,31 +19441,67 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F18" s="7" t="n"/>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="F33" s="7" t="n"/>
+      <c r="G33" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/en/missions/al-riyadh/contact-us/media-interview-request</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="351" customHeight="1">
-      <c r="A19" s="7" t="n">
-        <v>17</v>
-      </c>
-      <c r="B19" s="8" t="n">
+    <row r="34" ht="231" customHeight="1">
+      <c r="A34" s="7" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" s="8" t="n">
+        <v>46244</v>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>Request for Sitecore Path to Update Text – Doha Mission Contact Form</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srini,
+Thank you very much for your continued support and assistance.
+Could you please help me identify how I can update the highlighted text shown in the attached screenshot?
+I would appreciate it if you could advise me on the relevant Sitecore path or the correct location in the CMS where this text can be modified.
+Page URL:
+https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Doha/Contact-Form
+Please find the attached screenshot for reference.
+Thank you in advance for your support and guidance.</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Doha/Contact-Form</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="n"/>
+    </row>
+    <row r="35" ht="351" customHeight="1">
+      <c r="A35" s="7" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" s="8" t="n">
         <v>46245</v>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C35" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D35" s="7" t="inlineStr">
         <is>
           <t>Request for Official Image Dimensions – New Missions Template</t>
         </is>
       </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="E35" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 Thank you very much for your continued support and assistance.
@@ -18973,31 +19519,31 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F19" s="7" t="n"/>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="F35" s="7" t="n"/>
+      <c r="G35" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/en/Missions/_Inprogress/Abuja/The-Embassy/About-the-Ambassador</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="246" customHeight="1">
-      <c r="A20" s="7" t="n">
-        <v>18</v>
-      </c>
-      <c r="B20" s="8" t="n">
+    <row r="36" ht="246" customHeight="1">
+      <c r="A36" s="7" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" s="8" t="n">
         <v>46245</v>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C36" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D36" s="7" t="inlineStr">
         <is>
           <t>Request to Update the News Section Template – Oslo Mission Website</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E36" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 Thank you very much for your continued support and assistance.
@@ -19012,31 +19558,31 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="F36" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Oslo/Media-hub/News</t>
         </is>
       </c>
-      <c r="G20" s="7" t="n"/>
-    </row>
-    <row r="21" ht="261" customHeight="1">
-      <c r="A21" s="7" t="n">
-        <v>19</v>
-      </c>
-      <c r="B21" s="8" t="n">
+      <c r="G36" s="7" t="n"/>
+    </row>
+    <row r="37" ht="261" customHeight="1">
+      <c r="A37" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" s="8" t="n">
         <v>46245</v>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D37" s="7" t="inlineStr">
         <is>
           <t>Request to Update the News Section Template – Kuwait Mission Website</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="E37" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 Thank you very much for your continued support and assistance.
@@ -19051,31 +19597,31 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="F37" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/kuwait/Media-hub/News</t>
         </is>
       </c>
-      <c r="G21" s="7" t="n"/>
-    </row>
-    <row r="22" ht="276" customHeight="1">
-      <c r="A22" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="B22" s="8" t="n">
+      <c r="G37" s="7" t="n"/>
+    </row>
+    <row r="38" ht="276" customHeight="1">
+      <c r="A38" s="7" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" s="8" t="n">
         <v>46246</v>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C38" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D38" s="7" t="inlineStr">
         <is>
           <t>Request to Correct Arabic Labels on the New Missions Websites</t>
         </is>
       </c>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="E38" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 Please find attached two screenshots highlighting an issue with two Arabic labels displayed incorrectly on the new missions websites.
@@ -19093,31 +19639,31 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr">
+      <c r="F38" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/missions/cairo</t>
         </is>
       </c>
-      <c r="G22" s="7" t="n"/>
-    </row>
-    <row r="23" ht="381" customHeight="1">
-      <c r="A23" s="7" t="n">
-        <v>21</v>
-      </c>
-      <c r="B23" s="8" t="n">
+      <c r="G38" s="7" t="n"/>
+    </row>
+    <row r="39" ht="381" customHeight="1">
+      <c r="A39" s="7" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" s="8" t="n">
         <v>46246</v>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C39" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D39" s="7" t="inlineStr">
         <is>
           <t>Request to Update the News Section to the New Template – Maldives &amp; Muscat Missions</t>
         </is>
       </c>
-      <c r="E23" s="9" t="inlineStr">
+      <c r="E39" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 Thank you very much for your continued support and assistance.
@@ -19138,31 +19684,31 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
+      <c r="F39" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/male/Media-hub/News</t>
         </is>
       </c>
-      <c r="G23" s="7" t="n"/>
-    </row>
-    <row r="24" ht="261" customHeight="1">
-      <c r="A24" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="B24" s="8" t="n">
+      <c r="G39" s="7" t="n"/>
+    </row>
+    <row r="40" ht="261" customHeight="1">
+      <c r="A40" s="7" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" s="8" t="n">
         <v>46246</v>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C40" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D40" s="7" t="inlineStr">
         <is>
           <t>Request to Update Terminology Across Missions Websites</t>
         </is>
       </c>
-      <c r="E24" s="9" t="inlineStr">
+      <c r="E40" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 Based on a request from Nasra from the Government Communication Department, we kindly request your support in updating the following terminology across the missions websites.
@@ -19177,27 +19723,53 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F24" s="7" t="n"/>
-      <c r="G24" s="7" t="n"/>
-    </row>
-    <row r="25" ht="409" customHeight="1">
-      <c r="A25" s="7" t="n">
-        <v>23</v>
-      </c>
-      <c r="B25" s="8" t="n">
+      <c r="F40" s="7" t="n"/>
+      <c r="G40" s="7" t="n"/>
+    </row>
+    <row r="41" ht="51" customHeight="1">
+      <c r="A41" s="7" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" s="8" t="n">
+        <v>46246</v>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>Terminology Update (الكفيل) – Clarification on Scope</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="inlineStr">
+        <is>
+          <t>(Reply to Srini's question on whether the word includes the bracket or not)
+I will send to the ministry to ask them, as they have not specified the pages.</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="n"/>
+      <c r="G41" s="7" t="n"/>
+    </row>
+    <row r="42" ht="409" customHeight="1">
+      <c r="A42" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" s="8" t="n">
         <v>46247</v>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C42" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D42" s="7" t="inlineStr">
         <is>
           <t>Request to Update News Templates and Resolve German Language Issue – Kigali &amp; Bern Missions</t>
         </is>
       </c>
-      <c r="E25" s="9" t="inlineStr">
+      <c r="E42" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 Thank you very much for your continued support and assistance.
@@ -19228,31 +19800,118 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
+      <c r="F42" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/kigali</t>
         </is>
       </c>
-      <c r="G25" s="7" t="n"/>
-    </row>
-    <row r="26" ht="409" customHeight="1">
-      <c r="A26" s="7" t="n">
-        <v>24</v>
-      </c>
-      <c r="B26" s="8" t="n">
+      <c r="G42" s="7" t="n"/>
+    </row>
+    <row r="43" ht="111" customHeight="1">
+      <c r="A43" s="7" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" s="8" t="n">
+        <v>46247</v>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>CMS Hanging Issue – System Freezes for 10 to 15 Minutes</t>
+        </is>
+      </c>
+      <c r="E43" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srini, the team is facing this issue multiple times, the system hangs after this for 10 to 15 minutes and start working again, this happened at 10 today.
+It happens often but the guys were not reporting it.
+I asked them now to report it every time it happens.
+(Screenshots of the error attached)</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="n"/>
+      <c r="G43" s="7" t="n"/>
+    </row>
+    <row r="44" ht="171" customHeight="1">
+      <c r="A44" s="7" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" s="8" t="n">
+        <v>46247</v>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Error When Publishing a News Article Through the CMS</t>
+        </is>
+      </c>
+      <c r="E44" s="9" t="inlineStr">
+        <is>
+          <t>Thank you for your continued support.
+We are currently experiencing an issue while attempting to publish a news article through the CMS, and the following error message is appearing on our end.
+Could you please investigate and resolve this issue at your earliest convenience so that we can proceed with publishing the news article?
+Thank you for your support and assistance.
+(Screenshots of the error attached)</t>
+        </is>
+      </c>
+      <c r="F44" s="7" t="n"/>
+      <c r="G44" s="7" t="n"/>
+    </row>
+    <row r="45" ht="216" customHeight="1">
+      <c r="A45" s="7" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" s="8" t="n">
+        <v>46247</v>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Error When Removing the Meta Title – Social Media Channels Page (All Missions)</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srini
+When we try to remove the Meta Title from the Social Media Channels page, the following error message appears.
+We need your support in resolving this issue, as it appears to be affecting all missions. For example, we have encountered the same issue on the Muscat Mission website.
+Sitecore Path:
+/sitecore/content/LDSC/Home/Missions/_Inprogress/Muscat/Media hub/Social Media Channels
+Could you please check and advise on the required solution?</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="n"/>
+      <c r="G45" s="7" t="n"/>
+    </row>
+    <row r="46" ht="409" customHeight="1">
+      <c r="A46" s="7" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" s="8" t="n">
         <v>46250</v>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C46" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D46" s="7" t="inlineStr">
         <is>
           <t>Request to Update News Sections to the New Template – Multiple Missions</t>
         </is>
       </c>
-      <c r="E26" s="9" t="inlineStr">
+      <c r="E46" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 Thank you very much for your continued support and assistance.
@@ -19278,31 +19937,31 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F26" s="7" t="inlineStr">
+      <c r="F46" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Pretoria/Media-hub/News</t>
         </is>
       </c>
-      <c r="G26" s="7" t="n"/>
-    </row>
-    <row r="27" ht="336" customHeight="1">
-      <c r="A27" s="7" t="n">
-        <v>25</v>
-      </c>
-      <c r="B27" s="8" t="n">
+      <c r="G46" s="7" t="n"/>
+    </row>
+    <row r="47" ht="336" customHeight="1">
+      <c r="A47" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" s="8" t="n">
         <v>46250</v>
       </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="C47" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D27" s="7" t="inlineStr">
+      <c r="D47" s="7" t="inlineStr">
         <is>
           <t>Request to Move Mission Websites from STG to Production</t>
         </is>
       </c>
-      <c r="E27" s="9" t="inlineStr">
+      <c r="E47" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 We kindly request your help in moving the following mission websites from the Staging (STG) environment to the Production (Live) environment:
@@ -19321,27 +19980,68 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F27" s="7" t="n"/>
-      <c r="G27" s="7" t="n"/>
-    </row>
-    <row r="28" ht="381" customHeight="1">
-      <c r="A28" s="7" t="n">
-        <v>26</v>
-      </c>
-      <c r="B28" s="8" t="n">
+      <c r="F47" s="7" t="n"/>
+      <c r="G47" s="7" t="n"/>
+    </row>
+    <row r="48" ht="409" customHeight="1">
+      <c r="A48" s="7" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" s="8" t="n">
+        <v>46250</v>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>Request to Add Health Insurance Advisory to Travel Guidelines – All Countries (UAE Traveller)</t>
+        </is>
+      </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srini,
+We kindly request your support with the following update based on the instructions received from the UAE Traveller team.
+Please add the below health insurance advisory to the Travel Guidelines for all countries, in both the Arabic and English versions:
+Arabic:
+يُنصح بالحصول على تأمين صحي دولي ساري المفعول قبل السفر، لتغطية أي احتياجات صحية أو علاجية أثناء السفر.
+English:
+It is advised to obtain valid international health insurance before traveling to cover any medical or healthcare needs that may arise during the trip.
+UAE Traveller – Travel Guidelines Page:
+https://www.mofa.gov.ae/travel-updates
+Kindly ensure that the advisory is applied consistently across all countries listed under the Travel Guidelines, in both languages.
+Please find the attached screenshot for reference, indicating the section where the content should be displayed.
+We would appreciate your assistance in implementing this update and confirming once it has been applied successfully across all countries.
+Thank you very much for your continued support and cooperation.</t>
+        </is>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/travel-updates</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="n"/>
+    </row>
+    <row r="49" ht="381" customHeight="1">
+      <c r="A49" s="7" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" s="8" t="n">
         <v>46252</v>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C49" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="D49" s="7" t="inlineStr">
         <is>
           <t>Request to Update News Sections to the New Template – Hyderabad, Mumbai &amp; Moroni Missions</t>
         </is>
       </c>
-      <c r="E28" s="9" t="inlineStr">
+      <c r="E49" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 We kindly request your help in updating the News sections for the following missions from the old template/design to the new approved News template, consistent with the updated format currently used across the missions websites.
@@ -19360,31 +20060,31 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F28" s="7" t="inlineStr">
+      <c r="F49" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Hyderabad/Media-hub/Consulate-General-News</t>
         </is>
       </c>
-      <c r="G28" s="7" t="n"/>
-    </row>
-    <row r="29" ht="381" customHeight="1">
-      <c r="A29" s="7" t="n">
-        <v>27</v>
-      </c>
-      <c r="B29" s="8" t="n">
+      <c r="G49" s="7" t="n"/>
+    </row>
+    <row r="50" ht="381" customHeight="1">
+      <c r="A50" s="7" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" s="8" t="n">
         <v>46253</v>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C50" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="D50" s="7" t="inlineStr">
         <is>
           <t>Request to Update News Sections to the New Template – São Paulo, Dakar &amp; Istanbul Missions</t>
         </is>
       </c>
-      <c r="E29" s="9" t="inlineStr">
+      <c r="E50" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 We kindly request your help in converting the News sections from the old template to the new approved News template for the following mission websites:
@@ -19403,31 +20103,31 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F29" s="7" t="inlineStr">
+      <c r="F50" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Sao-Paulo/Media-hub/The-Consulate-News</t>
         </is>
       </c>
-      <c r="G29" s="7" t="n"/>
-    </row>
-    <row r="30" ht="141" customHeight="1">
-      <c r="A30" s="7" t="n">
-        <v>28</v>
-      </c>
-      <c r="B30" s="8" t="n">
+      <c r="G50" s="7" t="n"/>
+    </row>
+    <row r="51" ht="141" customHeight="1">
+      <c r="A51" s="7" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" s="8" t="n">
         <v>46254</v>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C51" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D30" s="7" t="inlineStr">
+      <c r="D51" s="7" t="inlineStr">
         <is>
           <t>Website issues- Urdu language</t>
         </is>
       </c>
-      <c r="E30" s="9" t="inlineStr">
+      <c r="E51" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan
 A website issue has been identified on UAE missions abroad page:
@@ -19437,27 +20137,27 @@
 Regards</t>
         </is>
       </c>
-      <c r="F30" s="7" t="n"/>
-      <c r="G30" s="7" t="n"/>
-    </row>
-    <row r="31" ht="306" customHeight="1">
-      <c r="A31" s="7" t="n">
-        <v>29</v>
-      </c>
-      <c r="B31" s="8" t="n">
+      <c r="F51" s="7" t="n"/>
+      <c r="G51" s="7" t="n"/>
+    </row>
+    <row r="52" ht="306" customHeight="1">
+      <c r="A52" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" s="8" t="n">
         <v>46254</v>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="C52" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D31" s="7" t="inlineStr">
+      <c r="D52" s="7" t="inlineStr">
         <is>
           <t>Request to Update News Sections to the New Template – Guangzhou &amp; Hong Kong Missions</t>
         </is>
       </c>
-      <c r="E31" s="9" t="inlineStr">
+      <c r="E52" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 We kindly request your help in converting the News sections from the old template to the new approved News template for the following mission websites:
@@ -19473,31 +20173,31 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F31" s="7" t="inlineStr">
+      <c r="F52" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Guangzhou/Media-hub/Embassy-News</t>
         </is>
       </c>
-      <c r="G31" s="7" t="n"/>
-    </row>
-    <row r="32" ht="321" customHeight="1">
-      <c r="A32" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="B32" s="8" t="n">
+      <c r="G52" s="7" t="n"/>
+    </row>
+    <row r="53" ht="321" customHeight="1">
+      <c r="A53" s="7" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" s="8" t="n">
         <v>46254</v>
       </c>
-      <c r="C32" s="7" t="inlineStr">
+      <c r="C53" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D32" s="7" t="inlineStr">
+      <c r="D53" s="7" t="inlineStr">
         <is>
           <t>Support Required: Urdu Text Direction (RTL) Issue – Karachi Mission Website</t>
         </is>
       </c>
-      <c r="E32" s="9" t="inlineStr">
+      <c r="E53" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 We are currently experiencing an issue with the Urdu language text direction on the Karachi Mission website. We need the Urdu content to be displayed correctly from right to left (RTL); however, we are unable to apply the required text direction properly.
@@ -19512,31 +20212,31 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F32" s="7" t="inlineStr">
+      <c r="F53" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ur-pk/missions/karachi-pakistan/services/digital-attestation</t>
         </is>
       </c>
-      <c r="G32" s="7" t="n"/>
-    </row>
-    <row r="33" ht="396" customHeight="1">
-      <c r="A33" s="7" t="n">
-        <v>31</v>
-      </c>
-      <c r="B33" s="8" t="n">
+      <c r="G53" s="7" t="n"/>
+    </row>
+    <row r="54" ht="396" customHeight="1">
+      <c r="A54" s="7" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" s="8" t="n">
         <v>46254</v>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C54" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D54" s="7" t="inlineStr">
         <is>
           <t>Issue with Date Display in Embassy Statements – Sofia Mission Website</t>
         </is>
       </c>
-      <c r="E33" s="9" t="inlineStr">
+      <c r="E54" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 We are currently experiencing an issue with the date display in the Embassy Statements section on the new Sofia Mission website.
@@ -19557,31 +20257,31 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F33" s="7" t="inlineStr">
+      <c r="F54" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/sofia</t>
         </is>
       </c>
-      <c r="G33" s="7" t="n"/>
-    </row>
-    <row r="34" ht="246" customHeight="1">
-      <c r="A34" s="7" t="n">
-        <v>32</v>
-      </c>
-      <c r="B34" s="8" t="n">
+      <c r="G54" s="7" t="n"/>
+    </row>
+    <row r="55" ht="246" customHeight="1">
+      <c r="A55" s="7" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" s="8" t="n">
         <v>46254</v>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C55" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D34" s="7" t="inlineStr">
+      <c r="D55" s="7" t="inlineStr">
         <is>
           <t>Re: Request to Update Terminology Across Missions Websites</t>
         </is>
       </c>
-      <c r="E34" s="9" t="inlineStr">
+      <c r="E55" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 We have a question regarding the search capabilities available within the CMS.
@@ -19593,27 +20293,56 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F34" s="7" t="n"/>
-      <c r="G34" s="7" t="n"/>
-    </row>
-    <row r="35" ht="409" customHeight="1">
-      <c r="A35" s="7" t="n">
-        <v>33</v>
-      </c>
-      <c r="B35" s="8" t="n">
+      <c r="F55" s="7" t="n"/>
+      <c r="G55" s="7" t="n"/>
+    </row>
+    <row r="56" ht="141" customHeight="1">
+      <c r="A56" s="7" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" s="8" t="n">
+        <v>46256</v>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>Recurring CMS Connection Error – Possible Network Issue (Azure / Du)</t>
+        </is>
+      </c>
+      <c r="E56" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srini, the team is experiencing this issue since the morning, like 4 times at least.
+We use Azure UAE virtual machine.
+Is it an issue with Azure network with Du?
+Do you have their email?
+(Screenshots of the error attached)</t>
+        </is>
+      </c>
+      <c r="F56" s="7" t="n"/>
+      <c r="G56" s="7" t="n"/>
+    </row>
+    <row r="57" ht="409" customHeight="1">
+      <c r="A57" s="7" t="n">
+        <v>55</v>
+      </c>
+      <c r="B57" s="8" t="n">
         <v>46257</v>
       </c>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="C57" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D35" s="7" t="inlineStr">
+      <c r="D57" s="7" t="inlineStr">
         <is>
           <t>Request to Update News Sections to the New Template – Multiple Missions</t>
         </is>
       </c>
-      <c r="E35" s="9" t="inlineStr">
+      <c r="E57" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 We kindly request your help in converting the News sections from the old template to the new approved News template for the following mission websites:
@@ -19643,35 +20372,35 @@
 Thank you once again for your continued support and cooperation.</t>
         </is>
       </c>
-      <c r="F35" s="7" t="inlineStr">
+      <c r="F57" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Moscow</t>
         </is>
       </c>
-      <c r="G35" s="7" t="inlineStr">
+      <c r="G57" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/en/missions/_inprogress/athens/media-hub/news</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="306" customHeight="1">
-      <c r="A36" s="7" t="n">
-        <v>34</v>
-      </c>
-      <c r="B36" s="8" t="n">
+    <row r="58" ht="306" customHeight="1">
+      <c r="A58" s="7" t="n">
+        <v>56</v>
+      </c>
+      <c r="B58" s="8" t="n">
         <v>46258</v>
       </c>
-      <c r="C36" s="7" t="inlineStr">
+      <c r="C58" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D36" s="7" t="inlineStr">
+      <c r="D58" s="7" t="inlineStr">
         <is>
           <t>Request to Update News Sections to the New Template – Madrid &amp; Victoria Missions</t>
         </is>
       </c>
-      <c r="E36" s="9" t="inlineStr">
+      <c r="E58" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 We kindly request your help in converting the News sections from the old template to the new approved News template for the following mission websites:
@@ -19687,31 +20416,31 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F36" s="7" t="inlineStr">
+      <c r="F58" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/madrid/Media-hub/News</t>
         </is>
       </c>
-      <c r="G36" s="7" t="n"/>
-    </row>
-    <row r="37" ht="409" customHeight="1">
-      <c r="A37" s="7" t="n">
-        <v>35</v>
-      </c>
-      <c r="B37" s="8" t="n">
+      <c r="G58" s="7" t="n"/>
+    </row>
+    <row r="59" ht="409" customHeight="1">
+      <c r="A59" s="7" t="n">
+        <v>57</v>
+      </c>
+      <c r="B59" s="8" t="n">
         <v>46259</v>
       </c>
-      <c r="C37" s="7" t="inlineStr">
+      <c r="C59" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D37" s="7" t="inlineStr">
+      <c r="D59" s="7" t="inlineStr">
         <is>
           <t>Request to Update News Sections to the New Template – Baku, Khartoum, Yerevan &amp; Tel Aviv Missions</t>
         </is>
       </c>
-      <c r="E37" s="9" t="inlineStr">
+      <c r="E59" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 We kindly request your help in converting the News sections from the old template to the new approved News template for the following mission websites:
@@ -19733,31 +20462,87 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F37" s="7" t="inlineStr">
+      <c r="F59" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/baku</t>
         </is>
       </c>
-      <c r="G37" s="7" t="n"/>
-    </row>
-    <row r="38" ht="409" customHeight="1">
-      <c r="A38" s="7" t="n">
-        <v>36</v>
-      </c>
-      <c r="B38" s="8" t="n">
+      <c r="G59" s="7" t="n"/>
+    </row>
+    <row r="60" ht="231" customHeight="1">
+      <c r="A60" s="7" t="n">
+        <v>58</v>
+      </c>
+      <c r="B60" s="8" t="n">
+        <v>46261</v>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>Follow-up: CMS Keyword Search Functionality (الكفيل)</t>
+        </is>
+      </c>
+      <c r="E60" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srini,
+I just wanted to kindly remind you regarding the email below, as we are still awaiting your response.
+Could you please advise whether there is any tool, functionality, or possible workaround within the CMS that could help us with this search requirement?
+Your feedback on this would be greatly appreciated.
+We need to search for the Arabic word "الكفيل".
+To clarify further, we do not have a specific path in mind. What we need is the ability to search across all pages of the missions' websites in general, to identify every location where a specific keyword appears.</t>
+        </is>
+      </c>
+      <c r="F60" s="7" t="n"/>
+      <c r="G60" s="7" t="n"/>
+    </row>
+    <row r="61" ht="66" customHeight="1">
+      <c r="A61" s="7" t="n">
+        <v>59</v>
+      </c>
+      <c r="B61" s="8" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>Urgent: Ministry Live Website and CMS Not Working</t>
+        </is>
+      </c>
+      <c r="E61" s="9" t="inlineStr">
+        <is>
+          <t>There is an issue with both the Ministry's live website and the CMS. Neither is working, and the following error messages are appearing.
+(Screenshots of the error messages attached)</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="n"/>
+      <c r="G61" s="7" t="n"/>
+    </row>
+    <row r="62" ht="409" customHeight="1">
+      <c r="A62" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="B62" s="8" t="n">
         <v>46264</v>
       </c>
-      <c r="C38" s="7" t="inlineStr">
+      <c r="C62" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D38" s="7" t="inlineStr">
+      <c r="D62" s="7" t="inlineStr">
         <is>
           <t>Request to Migrate News and Media Sections to the New Template – Multiple Missions</t>
         </is>
       </c>
-      <c r="E38" s="9" t="inlineStr">
+      <c r="E62" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 We kindly request your help in migrating the following News and Media sections from the old template to the new approved template across the missions listed below:
@@ -19783,31 +20568,31 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F38" s="7" t="inlineStr">
+      <c r="F62" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Lagos/Media-hub/Consulate-General-News</t>
         </is>
       </c>
-      <c r="G38" s="7" t="n"/>
-    </row>
-    <row r="39" ht="306" customHeight="1">
-      <c r="A39" s="7" t="n">
-        <v>37</v>
-      </c>
-      <c r="B39" s="8" t="n">
+      <c r="G62" s="7" t="n"/>
+    </row>
+    <row r="63" ht="306" customHeight="1">
+      <c r="A63" s="7" t="n">
+        <v>61</v>
+      </c>
+      <c r="B63" s="8" t="n">
         <v>46264</v>
       </c>
-      <c r="C39" s="7" t="inlineStr">
+      <c r="C63" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D39" s="7" t="inlineStr">
+      <c r="D63" s="7" t="inlineStr">
         <is>
           <t>500 Error When Accessing Arabic News Articles – Athens Mission</t>
         </is>
       </c>
-      <c r="E39" s="9" t="inlineStr">
+      <c r="E63" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 We would appreciate your assistance in investigating an issue affecting the Arabic News section of the Athens Mission website.
@@ -19823,31 +20608,31 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F39" s="7" t="inlineStr">
+      <c r="F63" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Athens/Media-hub/News</t>
         </is>
       </c>
-      <c r="G39" s="7" t="n"/>
-    </row>
-    <row r="40" ht="336" customHeight="1">
-      <c r="A40" s="7" t="n">
-        <v>38</v>
-      </c>
-      <c r="B40" s="8" t="n">
+      <c r="G63" s="7" t="n"/>
+    </row>
+    <row r="64" ht="336" customHeight="1">
+      <c r="A64" s="7" t="n">
+        <v>62</v>
+      </c>
+      <c r="B64" s="8" t="n">
         <v>46264</v>
       </c>
-      <c r="C40" s="7" t="inlineStr">
+      <c r="C64" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D40" s="7" t="inlineStr">
+      <c r="D64" s="7" t="inlineStr">
         <is>
           <t>Issue with Multiple Images and Video Not Displaying in Published News – Ashgabat Mission</t>
         </is>
       </c>
-      <c r="E40" s="9" t="inlineStr">
+      <c r="E64" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 We would appreciate your assistance in investigating an issue we encountered while publishing a news article on the Ashgabat Mission website.
@@ -19862,12 +20647,12 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F40" s="7" t="inlineStr">
+      <c r="F64" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/missions/_inprogress/ashgabat/media-hub/embassy-news/29-8-2026-1</t>
         </is>
       </c>
-      <c r="G40" s="7" t="n"/>
+      <c r="G64" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -19878,39 +20663,50 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId48"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>